<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 15:45
</commit_message>
<xml_diff>
--- a/Casino_Gaming_Equities.xlsx
+++ b/Casino_Gaming_Equities.xlsx
@@ -632,31 +632,31 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>36.68</v>
+        <v>37.57</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>10.032216064</v>
+        <v>10.275636224</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>39.510892544</v>
+        <v>39.71811328</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>0.155</v>
+        <v>0.189</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.005</v>
+        <v>0.03</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>48.26316</v>
+        <v>49.43421</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>15.359427</v>
+        <v>16.034245</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>16.781</v>
+        <v>16.869</v>
       </c>
       <c r="L2" s="2" t="n">
         <v>1.396</v>
@@ -668,7 +668,7 @@
         <v>25.3</v>
       </c>
       <c r="O2" s="4" t="n">
-        <v>-0.08699999999999999</v>
+        <v>-0.064</v>
       </c>
       <c r="P2" s="3" t="n">
         <v>16.2</v>
@@ -691,31 +691,31 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>53.68</v>
+        <v>52.4</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>36.294897664</v>
+        <v>35.429445632</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>48.603385856</v>
+        <v>48.932605952</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>0.269</v>
+        <v>0.327</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>-0.173</v>
+        <v>-0.192</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>56</v>
+        <v>52.2</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>22.842554</v>
+        <v>22.297874</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>14.285942</v>
+        <v>13.945294</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>10.722</v>
+        <v>10.795</v>
       </c>
       <c r="L3" s="2" t="n">
         <v>0.888</v>
@@ -727,7 +727,7 @@
         <v>30.18</v>
       </c>
       <c r="O3" s="4" t="n">
-        <v>-0.238</v>
+        <v>-0.256</v>
       </c>
       <c r="P3" s="3" t="n">
         <v>11</v>
@@ -750,31 +750,31 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>100.43</v>
+        <v>99.47</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>10.473170944</v>
+        <v>10.37305856</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>19.792420864</v>
+        <v>19.942465536</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>0.176</v>
+        <v>0.165</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-0.179</v>
+        <v>-0.187</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>39.3</v>
+        <v>33.2</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>31.984076</v>
+        <v>31.678343</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>16.791367</v>
+        <v>16.740803</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>11.313</v>
+        <v>11.398</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>1.034</v>
@@ -786,7 +786,7 @@
         <v>65.25</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>-0.255</v>
+        <v>-0.262</v>
       </c>
       <c r="P4" s="3" t="n">
         <v>6.5</v>
@@ -809,22 +809,22 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>28.06</v>
+        <v>26.89</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5.727268352</v>
+        <v>5.488462336</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>30.62779904</v>
+        <v>30.37543424</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>-0</v>
+        <v>-0.004</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.191</v>
+        <v>0.141</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>-25.8</v>
+        <v>-21.9</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -832,10 +832,10 @@
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>30.335135</v>
+        <v>26.208576</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>8.763</v>
+        <v>8.691000000000001</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>1.977</v>
@@ -847,7 +847,7 @@
         <v>17.86</v>
       </c>
       <c r="O5" s="4" t="n">
-        <v>-0.111</v>
+        <v>-0.149</v>
       </c>
       <c r="P5" s="3" t="n">
         <v>11</v>
@@ -870,22 +870,22 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>14.31</v>
+        <v>14.57</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1.911047168</v>
+        <v>1.945769088</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>12.39401984</v>
+        <v>12.438409216</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>-0.163</v>
+        <v>-0.149</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-0.036</v>
+        <v>-0.019</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>-18.2</v>
+        <v>-19.4</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -893,10 +893,10 @@
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>8.221634</v>
+        <v>8.419385999999999</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>17.161</v>
+        <v>17.223</v>
       </c>
       <c r="L6" s="2" t="n">
         <v>1.364</v>
@@ -908,7 +908,7 @@
         <v>11.65</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>-0.306</v>
+        <v>-0.293</v>
       </c>
       <c r="P6" s="3" t="n">
         <v>6.4</v>
@@ -931,31 +931,31 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>81.64</v>
+        <v>82.94</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>6.163183616</v>
+        <v>6.261323776</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>8.520010751999999</v>
+        <v>8.763850752</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>0.203</v>
+        <v>0.235</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-0.053</v>
+        <v>-0.035</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>22.5</v>
+        <v>19.9</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>3.6187944</v>
+        <v>3.6764185</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>10.020362</v>
+        <v>10.179922</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>7.094</v>
+        <v>7.297</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>1.22</v>
@@ -967,7 +967,7 @@
         <v>58.94</v>
       </c>
       <c r="O7" s="4" t="n">
-        <v>-0.092</v>
+        <v>-0.078</v>
       </c>
       <c r="P7" s="3" t="n">
         <v>3.9</v>
@@ -990,31 +990,31 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>57.84</v>
+        <v>55.74</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>5.947507712</v>
+        <v>5.7315712</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>6.833080832</v>
+        <v>6.88619776</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0.357</v>
+        <v>0.325</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.067</v>
+        <v>-0.09699999999999999</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>41.6</v>
+        <v>38.1</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>18.538462</v>
+        <v>17.865385</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>17.602324</v>
+        <v>16.963236</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>8.396000000000001</v>
+        <v>8.461</v>
       </c>
       <c r="L8" s="2" t="n">
         <v>1.453</v>
@@ -1026,7 +1026,7 @@
         <v>35.09</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>-0.162</v>
+        <v>-0.192</v>
       </c>
       <c r="P8" s="3" t="n">
         <v>2.1</v>
@@ -1049,31 +1049,31 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>86.36</v>
+        <v>87.56999999999999</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>6.021774336</v>
+        <v>6.103311872</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>11.061479424</v>
+        <v>11.120023552</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>-0.215</v>
+        <v>-0.218</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>-0.229</v>
+        <v>-0.218</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>-2.2</v>
+        <v>-2.9</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>16.325142</v>
+        <v>16.553875</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>11.630915</v>
+        <v>11.793877</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>11.562</v>
+        <v>11.623</v>
       </c>
       <c r="L9" s="2" t="n">
         <v>0.66</v>
@@ -1085,7 +1085,7 @@
         <v>80.23999999999999</v>
       </c>
       <c r="O9" s="4" t="n">
-        <v>-0.271</v>
+        <v>-0.261</v>
       </c>
       <c r="P9" s="3" t="n">
         <v>2.6</v>
@@ -1108,31 +1108,31 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>100.41</v>
+        <v>97.22</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>1.795945344</v>
+        <v>1.738888576</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>1.712775296</v>
+        <v>1.695962368</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>0.196</v>
+        <v>0.223</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.049</v>
+        <v>0.015</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>21.5</v>
+        <v>20.2</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>18.491714</v>
+        <v>17.904236</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>16.889824</v>
+        <v>16.353237</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>8.981</v>
+        <v>8.893000000000001</v>
       </c>
       <c r="L10" s="2" t="n">
         <v>1.376</v>
@@ -1144,7 +1144,7 @@
         <v>69.98999999999999</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>-0.118</v>
+        <v>-0.146</v>
       </c>
       <c r="P10" s="3" t="n">
         <v>1.4</v>
@@ -1167,22 +1167,22 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>27.6</v>
+        <v>26.42</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0.728607232</v>
+        <v>0.69745664</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>1.185720576</v>
+        <v>1.154019712</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0.095</v>
+        <v>-0.005</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0.011</v>
+        <v>-0.023</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>5</v>
+        <v>5.5</v>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
@@ -1190,10 +1190,10 @@
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>22.809917</v>
+        <v>21.83471</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>9.715</v>
+        <v>9.455</v>
       </c>
       <c r="L11" s="2" t="n">
         <v>1.412</v>
@@ -1205,7 +1205,7 @@
         <v>19.57</v>
       </c>
       <c r="O11" s="4" t="n">
-        <v>-0.157</v>
+        <v>-0.193</v>
       </c>
       <c r="P11" s="3" t="n">
         <v>1</v>
@@ -1228,22 +1228,22 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>2.61</v>
+        <v>2.28</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.094277104</v>
+        <v>0.0824974</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.595555136</v>
+        <v>0.57715008</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>-0.352</v>
+        <v>-0.461</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.044</v>
+        <v>-0.08800000000000001</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>-53.3</v>
+        <v>-52.4</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
@@ -1251,10 +1251,10 @@
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>-6.3658533</v>
+        <v>-5.5609756</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>12.968</v>
+        <v>12.524</v>
       </c>
       <c r="L12" s="2" t="n">
         <v>1.327</v>
@@ -1266,7 +1266,7 @@
         <v>2.02</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>-0.473</v>
+        <v>-0.539</v>
       </c>
       <c r="P12" s="3" t="n">
         <v>0.2</v>
@@ -1289,22 +1289,22 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>12.69</v>
+        <v>11.31</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.623867456</v>
+        <v>0.556023808</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>6.127169536</v>
+        <v>7.794639872</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>-0.248</v>
+        <v>-0.105</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>-0.237</v>
+        <v>-0.32</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>34.8</v>
+        <v>39.4</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="J13" s="2" t="n">
-        <v>-8.516778</v>
+        <v>-13.962963</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>18.942</v>
+        <v>22.644</v>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
@@ -1329,7 +1329,7 @@
         <v>8.455</v>
       </c>
       <c r="O13" s="4" t="n">
-        <v>-0.388</v>
+        <v>-0.455</v>
       </c>
       <c r="P13" s="3" t="n">
         <v>2.5</v>
@@ -1352,22 +1352,22 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>25.87</v>
+        <v>21.27</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.877375488</v>
+        <v>10.587621376</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>13.515968512</v>
+        <v>11.322156032</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>-0.317</v>
+        <v>-0.426</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>-0.275</v>
+        <v>-0.404</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>-31.9</v>
+        <v>-37.8</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
@@ -1375,10 +1375,10 @@
         </is>
       </c>
       <c r="J14" s="2" t="n">
-        <v>13.265647</v>
+        <v>10.928429</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>49.53</v>
+        <v>41.491</v>
       </c>
       <c r="L14" s="2" t="n">
         <v>1.682</v>
@@ -1387,10 +1387,10 @@
         <v>48.78</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>21.01</v>
+        <v>20.89</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>-0.47</v>
+        <v>-0.5639999999999999</v>
       </c>
       <c r="P14" s="3" t="n">
         <v>4.8</v>
@@ -1413,22 +1413,22 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>108.37</v>
+        <v>103.57</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>18.999713792</v>
+        <v>18.119817216</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>30.678474752</v>
+        <v>29.807222784</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>-0.5429999999999999</v>
+        <v>-0.5639999999999999</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-0.504</v>
+        <v>-0.525</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>-48</v>
+        <v>-60</v>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
@@ -1436,10 +1436,10 @@
         </is>
       </c>
       <c r="J15" s="2" t="n">
-        <v>10.0341015</v>
+        <v>9.729478</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>14.39</v>
+        <v>13.981</v>
       </c>
       <c r="L15" s="2" t="n">
         <v>1.177</v>
@@ -1451,7 +1451,7 @@
         <v>99.95999999999999</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>-0.655</v>
+        <v>-0.67</v>
       </c>
       <c r="P15" s="3" t="n">
         <v>13</v>
@@ -1474,10 +1474,10 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>20.25</v>
+        <v>21.45</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>4.713887232</v>
+        <v>4.9932288</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
@@ -1485,19 +1485,19 @@
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>0.893</v>
+        <v>0.9520000000000001</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.049</v>
+        <v>0.111</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>53.7</v>
+        <v>50.3</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>65.32258</v>
+        <v>69.19355</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>27.060255</v>
+        <v>28.751812</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
@@ -1514,7 +1514,7 @@
         <v>9.66</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>-0.106</v>
+        <v>-0.053</v>
       </c>
       <c r="P16" s="3" t="n">
         <v>0.7</v>
@@ -1537,31 +1537,31 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>18.66</v>
+        <v>18</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>5.5224576</v>
+        <v>5.3271296</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>5.301457408</v>
+        <v>5.256410112</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>-0.07099999999999999</v>
+        <v>-0.2</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-0.2</v>
+        <v>-0.228</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>-23</v>
+        <v>-30.1</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>51.833332</v>
+        <v>49.999996</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>22.827965</v>
+        <v>21.844957</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>10.447</v>
+        <v>10.358</v>
       </c>
       <c r="L17" s="2" t="n">
         <v>2.002</v>
@@ -1573,7 +1573,7 @@
         <v>15.725</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>-0.421</v>
+        <v>-0.441</v>
       </c>
       <c r="P17" s="3" t="n">
         <v>1</v>
@@ -1613,7 +1613,7 @@
         <v>-0.239</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>-283</v>
+        <v>-275.9</v>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
@@ -1667,31 +1667,31 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>11.29</v>
+        <v>11.09</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>0.939417664</v>
+        <v>0.90464736</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>1.244623104</v>
+        <v>1.242176128</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>0.15</v>
+        <v>0.083</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.006999999999999999</v>
+        <v>-0.025</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>0.4</v>
+        <v>-1.8</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>18.816666</v>
+        <v>18.483334</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>12.19183</v>
+        <v>11.975854</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>6.582</v>
+        <v>6.569</v>
       </c>
       <c r="L19" s="2" t="n">
         <v>1.07</v>
@@ -1703,7 +1703,7 @@
         <v>9.015000000000001</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>-0.152</v>
+        <v>-0.167</v>
       </c>
       <c r="P19" s="3" t="n">
         <v>0.7</v>
@@ -1726,31 +1726,31 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>5.59</v>
+        <v>5.53</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>2.183930112</v>
+        <v>2.249559808</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>12.896504832</v>
+        <v>12.774216704</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>-0.006999999999999999</v>
+        <v>0.024</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>-0.256</v>
+        <v>-0.264</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>16.2</v>
+        <v>5.6</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>12.152174</v>
+        <v>12.021739</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>7.0262322</v>
+        <v>6.9508166</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>11.293</v>
+        <v>10.592</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>0.603</v>
@@ -1762,7 +1762,7 @@
         <v>4.55</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>-0.449</v>
+        <v>-0.455</v>
       </c>
       <c r="P20" s="3" t="n">
         <v>4.5</v>
@@ -1934,37 +1934,37 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>36.68</v>
+        <v>37.57</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>10.032216064</v>
+        <v>10.275636224</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>39.510892544</v>
+        <v>39.71811328</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>48.26316</v>
+        <v>49.43421</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>15.359427</v>
+        <v>16.034245</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>16.781</v>
+        <v>16.869</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>2.253</v>
+        <v>2.265</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>3.8992243</v>
+        <v>3.9938345</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>0.5720377</v>
+        <v>0.58591753</v>
       </c>
       <c r="L2" s="3" t="n">
         <v>0.76</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>2.38811</v>
+        <v>2.34311</v>
       </c>
       <c r="N2" s="3" t="n">
         <v>63.763</v>
@@ -1982,31 +1982,31 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>53.68</v>
+        <v>52.4</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>36.294897664</v>
+        <v>35.429445632</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>48.603385856</v>
+        <v>48.932605952</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>22.842554</v>
+        <v>22.297874</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>14.285942</v>
+        <v>13.945294</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>10.722</v>
+        <v>10.795</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>3.734</v>
+        <v>3.759</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>22.784382</v>
+        <v>22.241087</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>2.788269</v>
+        <v>2.7217827</v>
       </c>
       <c r="L3" s="3" t="n">
         <v>2.35</v>
@@ -2030,37 +2030,37 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>100.43</v>
+        <v>99.47</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>10.473170944</v>
+        <v>10.37305856</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>19.792420864</v>
+        <v>19.942465536</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>31.984076</v>
+        <v>31.678343</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>16.791367</v>
+        <v>16.740803</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>11.313</v>
+        <v>11.398</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>2.773</v>
+        <v>2.794</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>-37.36235</v>
+        <v>-37.00521</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>1.4672573</v>
+        <v>1.4532318</v>
       </c>
       <c r="L4" s="3" t="n">
         <v>3.14</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>5.98105</v>
+        <v>5.94177</v>
       </c>
       <c r="N4" s="3" t="n">
         <v>68.834</v>
@@ -2078,13 +2078,13 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>28.06</v>
+        <v>26.89</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5.727268352</v>
+        <v>5.488462336</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>30.62779904</v>
+        <v>30.37543424</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -2092,25 +2092,25 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>30.335135</v>
+        <v>26.208576</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>8.763</v>
+        <v>8.691000000000001</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>2.667</v>
+        <v>2.645</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>1.6226219</v>
+        <v>1.5549644</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>0.49863034</v>
+        <v>0.47783932</v>
       </c>
       <c r="L5" s="3" t="n">
         <v>-2.42</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>0.925</v>
+        <v>1.026</v>
       </c>
       <c r="N5" s="3" t="n">
         <v>55.221</v>
@@ -2128,13 +2128,13 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>14.31</v>
+        <v>14.57</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1.911047168</v>
+        <v>1.945769088</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>12.39401984</v>
+        <v>12.438409216</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -2142,25 +2142,25 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>8.221634</v>
+        <v>8.419385999999999</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>17.161</v>
+        <v>17.223</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>1.78</v>
+        <v>1.787</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>0.9850622999999999</v>
+        <v>1.00296</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>0.2745363</v>
+        <v>0.27952436</v>
       </c>
       <c r="L6" s="3" t="n">
         <v>-5.83</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>1.74053</v>
+        <v>1.73053</v>
       </c>
       <c r="N6" s="3" t="n">
         <v>48.14</v>
@@ -2178,31 +2178,31 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>81.64</v>
+        <v>82.94</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>6.163183616</v>
+        <v>6.261323776</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>8.520010751999999</v>
+        <v>8.763850752</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>3.6187944</v>
+        <v>3.6764185</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>10.020362</v>
+        <v>10.179922</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>7.094</v>
+        <v>7.297</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>2.082</v>
+        <v>2.142</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>2.3901396</v>
+        <v>2.428199</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>1.5061584</v>
+        <v>1.530142</v>
       </c>
       <c r="L7" s="3" t="n">
         <v>22.56</v>
@@ -2226,31 +2226,31 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>57.84</v>
+        <v>55.74</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>5.947507712</v>
+        <v>5.7315712</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>6.833080832</v>
+        <v>6.88619776</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>18.538462</v>
+        <v>17.865385</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>17.602324</v>
+        <v>16.963236</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>8.396000000000001</v>
+        <v>8.461</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>3.397</v>
+        <v>3.423</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>16.19261</v>
+        <v>15.604704</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>2.9567776</v>
+        <v>2.8494256</v>
       </c>
       <c r="L8" s="3" t="n">
         <v>3.12</v>
@@ -2274,31 +2274,31 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>86.36</v>
+        <v>87.56999999999999</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>6.021774336</v>
+        <v>6.103311872</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>11.061479424</v>
+        <v>11.120023552</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>16.325142</v>
+        <v>16.553875</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>11.630915</v>
+        <v>11.793877</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>11.562</v>
+        <v>11.623</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>3.781</v>
+        <v>3.801</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>5.952988</v>
+        <v>6.036396</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>2.058093</v>
+        <v>2.0859604</v>
       </c>
       <c r="L9" s="3" t="n">
         <v>5.29</v>
@@ -2322,31 +2322,31 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>100.41</v>
+        <v>97.22</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>1.795945344</v>
+        <v>1.738888576</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>1.712775296</v>
+        <v>1.695962368</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>18.491714</v>
+        <v>17.904236</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>16.889824</v>
+        <v>16.353237</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>8.981</v>
+        <v>8.893000000000001</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>3.142</v>
+        <v>3.111</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>3.3276994</v>
+        <v>3.2219791</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>3.2945569</v>
+        <v>3.1898897</v>
       </c>
       <c r="L10" s="3" t="n">
         <v>5.43</v>
@@ -2370,13 +2370,13 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>27.6</v>
+        <v>26.42</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0.728607232</v>
+        <v>0.69745664</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>1.185720576</v>
+        <v>1.154019712</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -2384,19 +2384,19 @@
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>22.809917</v>
+        <v>21.83471</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>9.715</v>
+        <v>9.455</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>1.868</v>
+        <v>1.818</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>1.7170587</v>
+        <v>1.6436481</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>1.1475738</v>
+        <v>1.0985109</v>
       </c>
       <c r="L11" s="3" t="n">
         <v>-0.23</v>
@@ -2420,13 +2420,13 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>2.61</v>
+        <v>2.28</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.094277104</v>
+        <v>0.0824974</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.595555136</v>
+        <v>0.57715008</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -2434,22 +2434,22 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>-6.3658533</v>
+        <v>-5.5609756</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>12.968</v>
+        <v>12.524</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>1.97</v>
+        <v>1.909</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>6.641221</v>
+        <v>32.571426</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>0.31178766</v>
+        <v>0.27283052</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>-1.11</v>
+        <v>-1.12</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>-0.41</v>
@@ -2470,13 +2470,13 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>12.69</v>
+        <v>11.31</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.623867456</v>
+        <v>0.556023808</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>6.127169536</v>
+        <v>7.794639872</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -2484,28 +2484,28 @@
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>-8.516778</v>
+        <v>-13.962963</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>18.942</v>
+        <v>22.644</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>2.46</v>
+        <v>2.934</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>1.1954781</v>
+        <v>0.5517612</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>0.250468</v>
+        <v>0.20929217</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>-13.26</v>
+        <v>-12.45</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>-1.49</v>
+        <v>-0.8100000000000001</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>44.167</v>
+        <v>44.78</v>
       </c>
     </row>
     <row r="14">
@@ -2520,13 +2520,13 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>25.87</v>
+        <v>21.27</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.877375488</v>
+        <v>10.587621376</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>13.515968512</v>
+        <v>11.322156032</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -2534,25 +2534,25 @@
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>13.265647</v>
+        <v>10.928429</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>49.53</v>
+        <v>41.491</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>2.232</v>
+        <v>1.87</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>20.274296</v>
+        <v>16.66928</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>2.1269011</v>
+        <v>1.7487122</v>
       </c>
       <c r="L14" s="3" t="n">
         <v>-0.01</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>1.95015</v>
+        <v>1.9463</v>
       </c>
       <c r="N14" s="3" t="n">
         <v>12.216</v>
@@ -2570,13 +2570,13 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>108.37</v>
+        <v>103.57</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>18.999713792</v>
+        <v>18.119817216</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>30.678474752</v>
+        <v>29.807222784</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -2584,25 +2584,25 @@
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>10.0341015</v>
+        <v>9.729478</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>14.39</v>
+        <v>13.981</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>1.873</v>
+        <v>1.819</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>2.1010082</v>
+        <v>2.0079486</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>1.1597214</v>
+        <v>1.1060134</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>-1.74</v>
+        <v>-1.75</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>10.80017</v>
+        <v>10.64497</v>
       </c>
       <c r="N15" s="3" t="n">
         <v>92.559</v>
@@ -2620,10 +2620,10 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>20.25</v>
+        <v>21.45</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>4.713887232</v>
+        <v>4.9932288</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
@@ -2631,10 +2631,10 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>65.32258</v>
+        <v>69.19355</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>27.060255</v>
+        <v>28.751812</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -2647,16 +2647,16 @@
         </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>13.747454</v>
+        <v>14.562119</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>4.1552987</v>
+        <v>4.401539</v>
       </c>
       <c r="L16" s="3" t="n">
         <v>0.31</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.7483300000000001</v>
+        <v>0.74604</v>
       </c>
       <c r="N16" s="3" t="n">
         <v>11.838</v>
@@ -2674,37 +2674,37 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>18.66</v>
+        <v>18</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>5.5224576</v>
+        <v>5.3271296</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>5.301457408</v>
+        <v>5.256410112</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>51.833332</v>
+        <v>49.999996</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>22.827965</v>
+        <v>21.844957</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>10.447</v>
+        <v>10.358</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>4.11</v>
+        <v>4.075</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>4.971564</v>
+        <v>4.75748</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>4.2810907</v>
+        <v>4.1296697</v>
       </c>
       <c r="L17" s="3" t="n">
         <v>0.36</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>0.81741846</v>
+        <v>0.8239888</v>
       </c>
       <c r="N17" s="3" t="n">
         <v>4.293</v>
@@ -2790,31 +2790,31 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>11.29</v>
+        <v>11.09</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>0.939417664</v>
+        <v>0.90464736</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>1.244623104</v>
+        <v>1.242176128</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>18.816666</v>
+        <v>18.483334</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>12.19183</v>
+        <v>11.975854</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>6.582</v>
+        <v>6.569</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>3.4452243</v>
+        <v>3.384193</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>0.7058196</v>
+        <v>0.67969537</v>
       </c>
       <c r="L19" s="3" t="n">
         <v>0.6</v>
@@ -2838,31 +2838,31 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>5.59</v>
+        <v>5.53</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>2.183930112</v>
+        <v>2.249559808</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>12.896504832</v>
+        <v>12.774216704</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>12.152174</v>
+        <v>12.021739</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>7.0262322</v>
+        <v>6.9508166</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>11.293</v>
+        <v>10.592</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>2.498</v>
+        <v>2.474</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>-1.751802</v>
+        <v>-1.7329991</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>0.42297187</v>
+        <v>0.43568265</v>
       </c>
       <c r="L20" s="3" t="n">
         <v>0.46</v>
@@ -3724,7 +3724,7 @@
         <v>0.51523995</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.15188</v>
+        <v>0.15241</v>
       </c>
       <c r="H12" s="4" t="n">
         <v>-0.01112</v>
@@ -3733,44 +3733,34 @@
         <v>-0.13294</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>-1.4696201</v>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>-1.8681101</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>0.00328</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0.045923988</v>
-      </c>
-      <c r="M12" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N12" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>0.046085</v>
+      </c>
+      <c r="M12" s="3" t="n">
+        <v>0.00997</v>
+      </c>
+      <c r="N12" s="3" t="n">
+        <v>0.014096375</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.532207008</v>
+        <v>0.534599008</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>0.030929</v>
+        <v>0.04067</v>
       </c>
       <c r="Q12" s="2" t="n">
-        <v>3746.09</v>
-      </c>
-      <c r="R12" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="S12" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>21063.79</v>
+      </c>
+      <c r="R12" s="2" t="n">
+        <v>0.721</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>0.603</v>
       </c>
     </row>
     <row r="13">
@@ -3785,7 +3775,7 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>0.054</v>
+        <v>0.286</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -3798,46 +3788,46 @@
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0.5516</v>
+        <v>0.5986900000000001</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.12987</v>
+        <v>0.12956999</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0.046469998</v>
+        <v>-0.045900002</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>-0.1741</v>
+        <v>-0.26389998</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>-1.1563</v>
+        <v>-0.5564</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>0.00361</v>
+        <v>0.0021</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>0.323472</v>
+        <v>0.344231008</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>-0.072174</v>
+        <v>-0.0912</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>-0.210665504</v>
+        <v>0.738918656</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>5.66363904</v>
+        <v>6.46434816</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>0.160688992</v>
+        <v>0.798422976</v>
       </c>
       <c r="Q13" s="2" t="n">
-        <v>1085.198</v>
+        <v>254.019</v>
       </c>
       <c r="R13" s="2" t="n">
-        <v>0.6830000000000001</v>
+        <v>0.798</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>0.446</v>
+        <v>0.633</v>
       </c>
     </row>
     <row r="14">
@@ -4299,13 +4289,13 @@
         </is>
       </c>
       <c r="F20" s="4" t="n">
-        <v>0.36734</v>
+        <v>0.37937</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.22117001</v>
+        <v>0.23358</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>0.11319</v>
+        <v>0.16118999</v>
       </c>
       <c r="I20" s="4" t="n">
         <v>0.03584</v>
@@ -4316,23 +4306,19 @@
         </is>
       </c>
       <c r="K20" s="4" t="n">
-        <v>0.04816</v>
+        <v>0.05314</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>1.141964032</v>
-      </c>
-      <c r="M20" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N20" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>1.20605696</v>
+      </c>
+      <c r="M20" s="3" t="n">
+        <v>0.818115008</v>
+      </c>
+      <c r="N20" s="3" t="n">
+        <v>0.425185376</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>7.024941056</v>
+        <v>7.031579136</v>
       </c>
       <c r="P20" s="3" t="n">
         <v>1.023198976</v>
@@ -4469,7 +4455,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>36.68</v>
+        <v>37.57</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -4489,25 +4475,25 @@
         <v>31</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>42.61111</v>
+        <v>42.66667</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>42.5</v>
       </c>
       <c r="K2" s="8" t="n">
-        <v>22752018</v>
+        <v>23688418</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>4.2</v>
+        <v>4.85</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>0.1497</v>
+        <v>0.1559</v>
       </c>
       <c r="N2" s="4" t="n">
         <v>0.27018</v>
       </c>
       <c r="O2" s="4" t="n">
-        <v>0.73443</v>
+        <v>0.73356</v>
       </c>
     </row>
     <row r="3">
@@ -4522,7 +4508,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>53.68</v>
+        <v>52.4</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -4548,19 +4534,19 @@
         <v>71</v>
       </c>
       <c r="K3" s="8" t="n">
-        <v>11107798</v>
+        <v>10219140</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>1.8</v>
+        <v>2.49</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>0.034</v>
+        <v>0.0312</v>
       </c>
       <c r="N3" s="4" t="n">
         <v>0.57722</v>
       </c>
       <c r="O3" s="4" t="n">
-        <v>0.41689</v>
+        <v>0.41691002</v>
       </c>
     </row>
     <row r="4">
@@ -4575,7 +4561,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>100.43</v>
+        <v>99.47</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -4601,19 +4587,19 @@
         <v>143.5</v>
       </c>
       <c r="K4" s="8" t="n">
-        <v>5694412</v>
+        <v>6833602</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>3.24</v>
+        <v>3.38</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>0.0696</v>
+        <v>0.083500005</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>0.27027</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>0.68579</v>
+        <v>0.68557</v>
       </c>
     </row>
     <row r="5">
@@ -4628,7 +4614,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>28.06</v>
+        <v>26.89</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -4654,19 +4640,19 @@
         <v>33.62</v>
       </c>
       <c r="K5" s="8" t="n">
-        <v>30537844</v>
+        <v>26892014</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>3.8</v>
+        <v>3.37</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>0.1713</v>
+        <v>0.1509</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>0.02256</v>
+        <v>0.010570001</v>
       </c>
       <c r="O5" s="4" t="n">
-        <v>1.11971</v>
+        <v>1.1195099</v>
       </c>
     </row>
     <row r="6">
@@ -4681,7 +4667,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>14.31</v>
+        <v>14.57</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -4707,13 +4693,13 @@
         <v>20</v>
       </c>
       <c r="K6" s="8" t="n">
-        <v>21492483</v>
+        <v>21810886</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>4.18</v>
+        <v>4.3</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>0.16350001</v>
+        <v>0.1659</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>0.01867</v>
@@ -4734,7 +4720,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>81.64</v>
+        <v>82.94</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -4760,19 +4746,19 @@
         <v>93</v>
       </c>
       <c r="K7" s="8" t="n">
-        <v>3367790</v>
+        <v>3749544</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>3.32</v>
+        <v>3.91</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>0.0583</v>
+        <v>0.065</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>0.32334998</v>
+        <v>0.30977</v>
       </c>
       <c r="O7" s="4" t="n">
-        <v>0.7323499999999999</v>
+        <v>0.73407</v>
       </c>
     </row>
     <row r="8">
@@ -4787,7 +4773,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>57.84</v>
+        <v>55.74</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -4795,10 +4781,10 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>1.6</v>
+        <v>1.5625</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>80</v>
@@ -4807,25 +4793,25 @@
         <v>59</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>73.33333</v>
+        <v>72.9375</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>76</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>3025746</v>
+        <v>3346495</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>3.89</v>
+        <v>4.01</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>0.0762</v>
+        <v>0.084300004</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>0.07935</v>
+        <v>0.07914</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>0.889</v>
+        <v>0.88883</v>
       </c>
     </row>
     <row r="9">
@@ -4840,7 +4826,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>86.36</v>
+        <v>87.56999999999999</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -4866,19 +4852,19 @@
         <v>139.5</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>2574942</v>
+        <v>2415829</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>2.68</v>
+        <v>2.17</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>0.044499997</v>
+        <v>0.0368</v>
       </c>
       <c r="N9" s="4" t="n">
         <v>0.06136</v>
       </c>
       <c r="O9" s="4" t="n">
-        <v>0.83892995</v>
+        <v>0.81711</v>
       </c>
     </row>
     <row r="10">
@@ -4893,7 +4879,7 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>100.41</v>
+        <v>97.22</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -4921,19 +4907,19 @@
         <v>105.5</v>
       </c>
       <c r="K10" s="8" t="n">
-        <v>307491</v>
+        <v>289167</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>2.53</v>
+        <v>2.64</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>0.026199998</v>
+        <v>0.024600001</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>0.3204</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>0.64761</v>
+        <v>0.64763</v>
       </c>
     </row>
     <row r="11">
@@ -4948,15 +4934,17 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>27.6</v>
+        <v>26.42</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>hold</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>3</v>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="F11" s="2" t="n">
         <v>4</v>
@@ -4974,19 +4962,19 @@
         <v>30</v>
       </c>
       <c r="K11" s="8" t="n">
-        <v>640591</v>
+        <v>653244</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>2.5</v>
+        <v>4.41</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>0.0402</v>
+        <v>0.04</v>
       </c>
       <c r="N11" s="4" t="n">
         <v>0.27324</v>
       </c>
       <c r="O11" s="4" t="n">
-        <v>0.68558997</v>
+        <v>0.68551004</v>
       </c>
     </row>
     <row r="12">
@@ -5001,7 +4989,7 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>2.61</v>
+        <v>2.28</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
@@ -5027,19 +5015,19 @@
         <v>3.25</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>830872</v>
+        <v>771157</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>5.72</v>
+        <v>5.74</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>0.024300002</v>
+        <v>0.0225</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>0.0678</v>
+        <v>0.06769</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>0.40694</v>
+        <v>0.40625</v>
       </c>
     </row>
     <row r="13">
@@ -5054,7 +5042,7 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>12.69</v>
+        <v>11.31</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -5065,7 +5053,7 @@
         <v>3.2</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>18</v>
@@ -5074,25 +5062,25 @@
         <v>11</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>16.25</v>
+        <v>15.66667</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>18</v>
       </c>
       <c r="K13" s="8" t="n">
-        <v>825105</v>
+        <v>814259</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>9.16</v>
+        <v>8.01</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>0.1069</v>
+        <v>0.105500005</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>0.12553</v>
+        <v>0.12715</v>
       </c>
       <c r="O13" s="4" t="n">
-        <v>0.77327</v>
+        <v>0.78096</v>
       </c>
     </row>
     <row r="14">
@@ -5107,7 +5095,7 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>25.87</v>
+        <v>21.27</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
@@ -5115,7 +5103,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>1.54286</v>
+        <v>1.6</v>
       </c>
       <c r="F14" s="2" t="n">
         <v>34</v>
@@ -5127,25 +5115,25 @@
         <v>24</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>36.40882</v>
+        <v>36.17353</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>35</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>32087867</v>
+        <v>37514956</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>1.74</v>
+        <v>2.13</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>0.06670000399999999</v>
+        <v>0.078</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>0.02999</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>0.88236</v>
+        <v>0.88254</v>
       </c>
     </row>
     <row r="15">
@@ -5160,7 +5148,7 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>108.37</v>
+        <v>103.57</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
@@ -5180,25 +5168,25 @@
         <v>125</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>212.74074</v>
+        <v>207.44444</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="K15" s="8" t="n">
-        <v>9052256</v>
+        <v>10212758</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>1.72</v>
+        <v>2.02</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>0.0517</v>
+        <v>0.0583</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>0.18747</v>
+        <v>0.1886</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>0.90977997</v>
+        <v>0.91332</v>
       </c>
     </row>
     <row r="16">
@@ -5213,7 +5201,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>20.25</v>
+        <v>21.45</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -5224,7 +5212,7 @@
         <v>1.4</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>30</v>
@@ -5233,25 +5221,25 @@
         <v>20</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>24.8</v>
+        <v>24.90909</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>25</v>
       </c>
       <c r="K16" s="8" t="n">
-        <v>4779469</v>
+        <v>4216183</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>1.71</v>
+        <v>1.89</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>0.0498</v>
+        <v>0.043899998</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>0.07383000000000001</v>
+        <v>0.07084</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>0.93141997</v>
+        <v>0.93138003</v>
       </c>
     </row>
     <row r="17">
@@ -5266,7 +5254,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>18.66</v>
+        <v>18</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -5280,31 +5268,31 @@
         <v>21</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>36.745487</v>
+        <v>37.110058</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>21.673521</v>
+        <v>22.909552</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>28.490166</v>
+        <v>28.831713</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>27.583961</v>
+        <v>27.857635</v>
       </c>
       <c r="K17" s="8" t="n">
-        <v>11183802</v>
+        <v>10753999</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>4.19</v>
+        <v>4.54</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>0.1088</v>
+        <v>0.1046</v>
       </c>
       <c r="N17" s="4" t="n">
         <v>0.01337</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>0.9164</v>
+        <v>0.91643</v>
       </c>
     </row>
     <row r="18">
@@ -5394,7 +5382,7 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>11.29</v>
+        <v>11.09</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
@@ -5420,19 +5408,19 @@
         <v>16</v>
       </c>
       <c r="K19" s="8" t="n">
-        <v>1414201</v>
+        <v>1301175</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>3.68</v>
+        <v>2.55</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>0.028099999</v>
+        <v>0.0242</v>
       </c>
       <c r="N19" s="4" t="n">
-        <v>0.17429</v>
+        <v>0.13798</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>0.76091003</v>
+        <v>0.76087</v>
       </c>
     </row>
     <row r="20">
@@ -5447,7 +5435,7 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>5.59</v>
+        <v>5.53</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -5455,37 +5443,37 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>1.78571</v>
+        <v>1.84615</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G20" s="3" t="n">
         <v>12.3</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>6.4</v>
+        <v>6</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>9.625</v>
+        <v>9.24231</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>9.699999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>5850965</v>
+        <v>5741767</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>2.08</v>
+        <v>2.37</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>0.0388</v>
+        <v>0.0348</v>
       </c>
       <c r="N20" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>0.33803</v>
+        <v>0.32467</v>
       </c>
     </row>
   </sheetData>
@@ -5608,43 +5596,43 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>36.68</v>
+        <v>37.57</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>36.84</v>
+        <v>37.59</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>37.43</v>
+        <v>37.97</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>36.454</v>
+        <v>36.9</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>36.3</v>
+        <v>37.49</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>0.380001</v>
+        <v>0.079998</v>
       </c>
       <c r="I2" s="9" t="n">
-        <v>1.04683</v>
+        <v>0.213385</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>35.3842</v>
+        <v>35.4426</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>35.0487</v>
+        <v>35.16575</v>
       </c>
       <c r="L2" s="8" t="n">
-        <v>4927380</v>
+        <v>5265930</v>
       </c>
       <c r="M2" s="8" t="n">
-        <v>4763773</v>
+        <v>4897876</v>
       </c>
       <c r="N2" s="3" t="n">
         <v>0.76</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>2.38811</v>
+        <v>2.34311</v>
       </c>
     </row>
     <row r="3">
@@ -5659,37 +5647,37 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>53.68</v>
+        <v>52.4</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>54.12</v>
+        <v>53.62</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>54.465</v>
+        <v>53.94</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>53.37</v>
+        <v>52.01</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>53.68</v>
+        <v>54.17</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>0</v>
+        <v>-1.77</v>
       </c>
       <c r="I3" s="9" t="n">
-        <v>0</v>
+        <v>-3.26749</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>57.902</v>
+        <v>56.8742</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>55.40065</v>
+        <v>55.7133</v>
       </c>
       <c r="L3" s="8" t="n">
-        <v>3730880</v>
+        <v>3958140</v>
       </c>
       <c r="M3" s="8" t="n">
-        <v>5519521</v>
+        <v>5419925</v>
       </c>
       <c r="N3" s="3" t="n">
         <v>2.35</v>
@@ -5710,43 +5698,43 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>100.43</v>
+        <v>99.47</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>100.21</v>
+        <v>100.86</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>101.7899</v>
+        <v>101.42</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>99.5</v>
+        <v>99.06999999999999</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>98.79000000000001</v>
+        <v>101.89</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>1.64</v>
+        <v>-2.4199982</v>
       </c>
       <c r="I4" s="9" t="n">
-        <v>1.66009</v>
+        <v>-2.3751085</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>111.7172</v>
+        <v>109.902</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>114.02265</v>
+        <v>114.32745</v>
       </c>
       <c r="L4" s="8" t="n">
-        <v>2562290</v>
+        <v>2163700</v>
       </c>
       <c r="M4" s="8" t="n">
-        <v>1633747</v>
+        <v>1655030</v>
       </c>
       <c r="N4" s="3" t="n">
         <v>3.14</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>5.98105</v>
+        <v>5.94177</v>
       </c>
     </row>
     <row r="5">
@@ -5761,43 +5749,43 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>28.06</v>
+        <v>26.89</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>28.39</v>
+        <v>26.48</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>28.68</v>
+        <v>27.02</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>27.81</v>
+        <v>26.3367</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>28.41</v>
+        <v>26.82</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>-0.35</v>
+        <v>0.069999695</v>
       </c>
       <c r="I5" s="9" t="n">
-        <v>-1.23196</v>
+        <v>0.26099813</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>23.0774</v>
+        <v>23.4482</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>24.655275</v>
+        <v>24.664825</v>
       </c>
       <c r="L5" s="8" t="n">
-        <v>6430020</v>
+        <v>6358500</v>
       </c>
       <c r="M5" s="8" t="n">
-        <v>6293229</v>
+        <v>6234857</v>
       </c>
       <c r="N5" s="3" t="n">
         <v>-2.42</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>0.925</v>
+        <v>1.026</v>
       </c>
     </row>
     <row r="6">
@@ -5812,43 +5800,43 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>14.31</v>
+        <v>14.57</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>14.75</v>
+        <v>14.51</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>15</v>
+        <v>14.97</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>14.3</v>
+        <v>14.445</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>14.53</v>
+        <v>14.66</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>-0.219999</v>
+        <v>-0.09000015</v>
       </c>
       <c r="I6" s="9" t="n">
-        <v>-1.5141</v>
+        <v>-0.61391646</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>13.8534</v>
+        <v>13.7784</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>16.2736</v>
+        <v>16.2453</v>
       </c>
       <c r="L6" s="8" t="n">
-        <v>4547870</v>
+        <v>4084830</v>
       </c>
       <c r="M6" s="8" t="n">
-        <v>4482001</v>
+        <v>4456361</v>
       </c>
       <c r="N6" s="3" t="n">
         <v>-5.83</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>1.74053</v>
+        <v>1.73053</v>
       </c>
     </row>
     <row r="7">
@@ -5863,37 +5851,37 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>81.64</v>
+        <v>82.94</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>81.7</v>
+        <v>84.44</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>82.23999999999999</v>
+        <v>85.13249999999999</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>80.90000000000001</v>
+        <v>82.86</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>81.3</v>
+        <v>84.87</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.339996</v>
+        <v>-1.93</v>
       </c>
       <c r="I7" s="9" t="n">
-        <v>0.4182</v>
+        <v>-2.27407</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>84.4358</v>
+        <v>83.916</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>82.6203</v>
+        <v>82.78945</v>
       </c>
       <c r="L7" s="8" t="n">
-        <v>1037530</v>
+        <v>1090120</v>
       </c>
       <c r="M7" s="8" t="n">
-        <v>916393</v>
+        <v>904479</v>
       </c>
       <c r="N7" s="3" t="n">
         <v>22.56</v>
@@ -5914,37 +5902,37 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>57.84</v>
+        <v>55.74</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>57.91</v>
+        <v>58.01</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>58.54</v>
+        <v>58.71</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>57.5</v>
+        <v>55.68</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>57.71</v>
+        <v>58.75</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.130001</v>
+        <v>-3.0099983</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>0.225266</v>
+        <v>-5.1234016</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>61.9843</v>
+        <v>61.6271</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>58.468925</v>
+        <v>58.705875</v>
       </c>
       <c r="L8" s="8" t="n">
-        <v>921060</v>
+        <v>941430</v>
       </c>
       <c r="M8" s="8" t="n">
-        <v>723195</v>
+        <v>727440</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>3.12</v>
@@ -5965,37 +5953,37 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>86.36</v>
+        <v>87.56999999999999</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>84.31999999999999</v>
+        <v>86.97</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>86.38</v>
+        <v>89.61</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>83.42</v>
+        <v>86.43000000000001</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>84.08</v>
+        <v>87.2</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>2.28</v>
+        <v>0.37000275</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>2.7117</v>
+        <v>0.4243151</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>97.4666</v>
+        <v>94.80240000000001</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>101.16975</v>
+        <v>100.96005</v>
       </c>
       <c r="L9" s="8" t="n">
-        <v>1255360</v>
+        <v>1091240</v>
       </c>
       <c r="M9" s="8" t="n">
-        <v>889204</v>
+        <v>909450</v>
       </c>
       <c r="N9" s="3" t="n">
         <v>5.29</v>
@@ -6016,37 +6004,37 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>100.41</v>
+        <v>97.22</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>100.4</v>
+        <v>99.56</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>102.84</v>
+        <v>100.325</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>99.77500000000001</v>
+        <v>96.97</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>99.66</v>
+        <v>99.47</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.75</v>
+        <v>-2.25</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>0.752559</v>
+        <v>-2.2619884</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>94.654</v>
+        <v>94.8856</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>95.79949999999999</v>
+        <v>96.1313</v>
       </c>
       <c r="L10" s="8" t="n">
-        <v>133860</v>
+        <v>158160</v>
       </c>
       <c r="M10" s="8" t="n">
-        <v>104962</v>
+        <v>110723</v>
       </c>
       <c r="N10" s="3" t="n">
         <v>5.43</v>
@@ -6067,37 +6055,37 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>27.6</v>
+        <v>26.42</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>27.79</v>
+        <v>26.38</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>28</v>
+        <v>26.66</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>27.5514</v>
+        <v>26.35</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>27.64</v>
+        <v>26.39</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>-0.039999</v>
+        <v>0.030000687</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>-0.144714</v>
+        <v>0.11368203</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>27.9474</v>
+        <v>27.9432</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>26.90945</v>
+        <v>26.87835</v>
       </c>
       <c r="L11" s="8" t="n">
-        <v>129150</v>
+        <v>143220</v>
       </c>
       <c r="M11" s="8" t="n">
-        <v>238147</v>
+        <v>232520</v>
       </c>
       <c r="N11" s="3" t="n">
         <v>-0.23</v>
@@ -6118,40 +6106,40 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>2.61</v>
+        <v>2.28</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>2.8845</v>
+        <v>2.28</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2.8845</v>
+        <v>2.3</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>2.5924</v>
+        <v>2.245</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>2.74</v>
+        <v>2.3</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>-0.13</v>
+        <v>-0.01999998</v>
       </c>
       <c r="I12" s="9" t="n">
-        <v>-4.74453</v>
+        <v>-0.8695644</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>2.425</v>
+        <v>2.415</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>3.1002</v>
+        <v>3.0828</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>174160</v>
+        <v>112720</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>160350</v>
+        <v>142789</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>-1.11</v>
+        <v>-1.12</v>
       </c>
       <c r="O12" s="3" t="n">
         <v>-0.41</v>
@@ -6169,43 +6157,43 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>12.69</v>
+        <v>11.31</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>13.01</v>
+        <v>11.74</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>13.365</v>
+        <v>11.97</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>12.48</v>
+        <v>11.31</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>13.03</v>
+        <v>11.92</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>-0.34</v>
+        <v>-0.61</v>
       </c>
       <c r="I13" s="9" t="n">
-        <v>-2.60936</v>
+        <v>-5.11745</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>14.9646</v>
+        <v>14.5238</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>13.2249</v>
+        <v>13.29165</v>
       </c>
       <c r="L13" s="8" t="n">
-        <v>121900</v>
+        <v>107850</v>
       </c>
       <c r="M13" s="8" t="n">
-        <v>97855</v>
+        <v>87925</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>-13.26</v>
+        <v>-12.45</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>-1.49</v>
+        <v>-0.8100000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -6220,43 +6208,43 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>25.87</v>
+        <v>21.27</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>25.75</v>
+        <v>21.1</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>26.46</v>
+        <v>21.63</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>25.6</v>
+        <v>20.89</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>25.54</v>
+        <v>21.42</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.33</v>
+        <v>-0.14999962</v>
       </c>
       <c r="I14" s="9" t="n">
-        <v>1.29209</v>
+        <v>-0.70027834</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>28.1998</v>
+        <v>27.1599</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>35.971973</v>
+        <v>35.7191</v>
       </c>
       <c r="L14" s="8" t="n">
-        <v>14780350</v>
+        <v>13781570</v>
       </c>
       <c r="M14" s="8" t="n">
-        <v>14439654</v>
+        <v>14937996</v>
       </c>
       <c r="N14" s="3" t="n">
         <v>-0.01</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>1.95015</v>
+        <v>1.9463</v>
       </c>
     </row>
     <row r="15">
@@ -6271,43 +6259,43 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>108.37</v>
+        <v>103.57</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>107.11</v>
+        <v>102.22</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>110.1</v>
+        <v>105.23</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>106.5</v>
+        <v>102.01</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>105.53</v>
+        <v>103.4</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>2.84</v>
+        <v>0.169998</v>
       </c>
       <c r="I15" s="9" t="n">
-        <v>2.69118</v>
+        <v>0.164408</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>154.8922</v>
+        <v>143.885</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>233.48535</v>
+        <v>229.95735</v>
       </c>
       <c r="L15" s="8" t="n">
-        <v>4034930</v>
+        <v>3297370</v>
       </c>
       <c r="M15" s="8" t="n">
-        <v>3833347</v>
+        <v>3929393</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>-1.74</v>
+        <v>-1.75</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>10.80017</v>
+        <v>10.64497</v>
       </c>
     </row>
     <row r="16">
@@ -6322,43 +6310,43 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>20.25</v>
+        <v>21.45</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>21</v>
+        <v>21.92</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>21.115</v>
+        <v>22.22</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>20.05</v>
+        <v>21.45</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>20.83</v>
+        <v>21.92</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>-0.58</v>
+        <v>-0.469999</v>
       </c>
       <c r="I16" s="9" t="n">
-        <v>-2.78445</v>
+        <v>-2.14416</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>18.6776</v>
+        <v>18.8108</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>18.08495</v>
+        <v>18.28475</v>
       </c>
       <c r="L16" s="8" t="n">
-        <v>1500550</v>
+        <v>1505260</v>
       </c>
       <c r="M16" s="8" t="n">
-        <v>2026744</v>
+        <v>2031306</v>
       </c>
       <c r="N16" s="3" t="n">
         <v>0.31</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.7483300000000001</v>
+        <v>0.74604</v>
       </c>
     </row>
     <row r="17">
@@ -6373,43 +6361,43 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>18.66</v>
+        <v>18</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>18.92</v>
+        <v>18.4501</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>18.92</v>
+        <v>18.975</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>18.33</v>
+        <v>17.605</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>19.12</v>
+        <v>18.51</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>-0.460001</v>
+        <v>-0.5100002</v>
       </c>
       <c r="I17" s="9" t="n">
-        <v>-2.40586</v>
+        <v>-2.7552686</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>18.762</v>
+        <v>18.3774</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>24.642025</v>
+        <v>24.513975</v>
       </c>
       <c r="L17" s="8" t="n">
-        <v>2877430</v>
+        <v>2485880</v>
       </c>
       <c r="M17" s="8" t="n">
-        <v>2490290</v>
+        <v>2657188</v>
       </c>
       <c r="N17" s="3" t="n">
         <v>0.36</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>0.81741846</v>
+        <v>0.8239888</v>
       </c>
     </row>
     <row r="18">
@@ -6493,37 +6481,37 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
+        <v>11.09</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>11.21</v>
+      </c>
+      <c r="E19" s="3" t="n">
         <v>11.29</v>
       </c>
-      <c r="D19" s="3" t="n">
-        <v>11.345</v>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>11.5</v>
-      </c>
       <c r="F19" s="3" t="n">
-        <v>11.23</v>
+        <v>11.0201</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>11.32</v>
+        <v>11.26</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>-0.0299997</v>
+        <v>-0.17</v>
       </c>
       <c r="I19" s="9" t="n">
-        <v>-0.265015</v>
+        <v>-1.50977</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>11.342</v>
+        <v>11.2952</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>11.20465</v>
+        <v>11.19845</v>
       </c>
       <c r="L19" s="8" t="n">
-        <v>646330</v>
+        <v>453170</v>
       </c>
       <c r="M19" s="8" t="n">
-        <v>444170</v>
+        <v>417416</v>
       </c>
       <c r="N19" s="3" t="n">
         <v>0.6</v>
@@ -6544,37 +6532,37 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>5.59</v>
+        <v>5.53</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>5.56</v>
+        <v>5.42</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>5.655</v>
+        <v>5.5801</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>5.495</v>
+        <v>5.4</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>5.5</v>
+        <v>5.48</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>0.0900002</v>
+        <v>0.05000019</v>
       </c>
       <c r="I20" s="9" t="n">
-        <v>1.63637</v>
+        <v>0.9124123</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>6.205</v>
+        <v>6.0186</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>7.86995</v>
+        <v>7.85155</v>
       </c>
       <c r="L20" s="8" t="n">
-        <v>2234280</v>
+        <v>1478700</v>
       </c>
       <c r="M20" s="8" t="n">
-        <v>2307352</v>
+        <v>2330632</v>
       </c>
       <c r="N20" s="3" t="n">
         <v>0.46</v>
@@ -6649,10 +6637,10 @@
         </is>
       </c>
       <c r="C2" s="11" t="n">
-        <v>0.893</v>
+        <v>0.9520000000000001</v>
       </c>
       <c r="D2" s="10" t="n">
-        <v>53.7</v>
+        <v>50.3</v>
       </c>
       <c r="E2" s="12" t="inlineStr">
         <is>
@@ -6664,19 +6652,19 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>RRR</t>
+          <t>LVS</t>
         </is>
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Red Rock Resorts, Inc.</t>
+          <t>Las Vegas Sands Corp.</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>0.357</v>
+        <v>0.327</v>
       </c>
       <c r="D3" s="10" t="n">
-        <v>41.6</v>
+        <v>52.2</v>
       </c>
       <c r="E3" s="12" t="inlineStr">
         <is>
@@ -6688,19 +6676,19 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>LVS</t>
+          <t>RRR</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>Las Vegas Sands Corp.</t>
+          <t>Red Rock Resorts, Inc.</t>
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>0.269</v>
+        <v>0.325</v>
       </c>
       <c r="D4" s="10" t="n">
-        <v>56</v>
+        <v>38.1</v>
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
@@ -6721,10 +6709,10 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>0.203</v>
+        <v>0.235</v>
       </c>
       <c r="D5" s="10" t="n">
-        <v>22.5</v>
+        <v>19.9</v>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
@@ -6736,23 +6724,23 @@
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>CHDN</t>
+          <t>MCRI</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Churchill Downs Incorporated</t>
+          <t>Monarch Casino &amp; Resort, Inc.</t>
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>-0.215</v>
+        <v>0.223</v>
       </c>
       <c r="D6" s="10" t="n">
-        <v>-2.2</v>
-      </c>
-      <c r="E6" s="13" t="inlineStr">
-        <is>
-          <t>Loser</t>
+        <v>20.2</v>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>Gainer</t>
         </is>
       </c>
       <c r="F6" s="10" t="n"/>
@@ -6760,19 +6748,19 @@
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>LNW</t>
+          <t>CHDN</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Light &amp; Wonder, Inc.</t>
+          <t>Churchill Downs Incorporated</t>
         </is>
       </c>
       <c r="C7" s="11" t="n">
-        <v>-0.239</v>
+        <v>-0.218</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>-283</v>
+        <v>-2.9</v>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
@@ -6784,19 +6772,19 @@
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>BALY</t>
+          <t>LNW</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>Bally's Corporation</t>
+          <t>Light &amp; Wonder, Inc.</t>
         </is>
       </c>
       <c r="C8" s="11" t="n">
-        <v>-0.248</v>
+        <v>-0.239</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>34.8</v>
+        <v>-275.9</v>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
@@ -6817,10 +6805,10 @@
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>-0.317</v>
+        <v>-0.426</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>-31.9</v>
+        <v>-37.8</v>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
@@ -6841,10 +6829,10 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>-0.352</v>
+        <v>-0.461</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>-53.3</v>
+        <v>-52.4</v>
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
@@ -6865,10 +6853,10 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>-0.5429999999999999</v>
+        <v>-0.5639999999999999</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>-48</v>
+        <v>-60</v>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
@@ -6953,19 +6941,19 @@
         <v>4</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>15.631888256</v>
+        <v>15.391650688</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>34.633624576</v>
+        <v>34.742154752</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>34.36326333333333</v>
+        <v>34.47014233333334</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>11.89475</v>
+        <v>11.93825</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.15</v>
+        <v>0.16925</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>44.7</v>
@@ -6981,19 +6969,19 @@
         <v>2</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>0.469708832</v>
+        <v>0.45232368</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1.244623104</v>
+        <v>1.242176128</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>18.816666</v>
+        <v>18.483334</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>6.582</v>
+        <v>6.569</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>-0.04449999999999999</v>
+        <v>-0.07799999999999999</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>3.6</v>
@@ -7009,19 +6997,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>2.183930112</v>
+        <v>2.249559808</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>12.896504832</v>
+        <v>12.774216704</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>12.152174</v>
+        <v>12.021739</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>11.293</v>
+        <v>10.592</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-0.006999999999999999</v>
+        <v>0.024</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>4.5</v>
@@ -7037,19 +7025,19 @@
         <v>4</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>10.528358528</v>
+        <v>9.756949248</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>16.49863355733333</v>
+        <v>15.46192964266667</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>58.577956</v>
+        <v>59.596773</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>24.789</v>
+        <v>21.94333333333333</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-0.009500000000000007</v>
+        <v>-0.05949999999999999</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>19.5</v>
@@ -7065,19 +7053,19 @@
         <v>8</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>2.910776246</v>
+        <v>2.889605295</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>6.053726424</v>
+        <v>6.303781664</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>14.2435281</v>
+        <v>13.999978625</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>11.852375</v>
+        <v>12.265</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-0.015875</v>
+        <v>-0.019375</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>20.1</v>
@@ -7130,7 +7118,7 @@
         </is>
       </c>
       <c r="B3" s="17" t="n">
-        <v>131.05054488</v>
+        <v>126.865449272</v>
       </c>
     </row>
     <row r="4">
@@ -7140,7 +7128,7 @@
         </is>
       </c>
       <c r="B4" s="17" t="n">
-        <v>250.601338304</v>
+        <v>249.80105408</v>
       </c>
     </row>
     <row r="5">
@@ -7150,7 +7138,7 @@
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>5.5224576</v>
+        <v>5.3271296</v>
       </c>
     </row>
     <row r="6">
@@ -7174,7 +7162,7 @@
         </is>
       </c>
       <c r="B8" s="18" t="n">
-        <v>28.0171504</v>
+        <v>28.10081459090909</v>
       </c>
     </row>
     <row r="9">
@@ -7184,7 +7172,7 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>18.816666</v>
+        <v>18.483334</v>
       </c>
     </row>
     <row r="10">
@@ -7194,7 +7182,7 @@
         </is>
       </c>
       <c r="B10" s="18" t="n">
-        <v>13.80235294117647</v>
+        <v>13.46258823529412</v>
       </c>
     </row>
     <row r="11">
@@ -7204,7 +7192,7 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>11.293</v>
+        <v>10.795</v>
       </c>
     </row>
     <row r="12">
@@ -7229,7 +7217,7 @@
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>Rush Street Interactive, Inc. (+89.3%)</t>
+          <t>Rush Street Interactive, Inc. (+95.2%)</t>
         </is>
       </c>
     </row>
@@ -7241,7 +7229,7 @@
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>Flutter Entertainment plc (-54.3%)</t>
+          <t>Flutter Entertainment plc (-56.4%)</t>
         </is>
       </c>
     </row>
@@ -7312,19 +7300,19 @@
         </is>
       </c>
       <c r="B2" s="19" t="n">
-        <v>36.68</v>
+        <v>37.57</v>
       </c>
       <c r="C2" s="20" t="n">
-        <v>0.155</v>
+        <v>0.189</v>
       </c>
       <c r="D2" s="20" t="n">
-        <v>0.005</v>
+        <v>0.03</v>
       </c>
       <c r="E2" s="16" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="F2" s="20" t="n">
-        <v>-0.08699999999999999</v>
+        <v>-0.064</v>
       </c>
       <c r="G2" s="16" t="n">
         <v>1.396</v>
@@ -7337,19 +7325,19 @@
         </is>
       </c>
       <c r="B3" s="19" t="n">
-        <v>53.68</v>
+        <v>52.4</v>
       </c>
       <c r="C3" s="20" t="n">
-        <v>0.269</v>
+        <v>0.327</v>
       </c>
       <c r="D3" s="20" t="n">
-        <v>-0.173</v>
+        <v>-0.192</v>
       </c>
       <c r="E3" s="16" t="n">
-        <v>56</v>
+        <v>52.2</v>
       </c>
       <c r="F3" s="20" t="n">
-        <v>-0.238</v>
+        <v>-0.256</v>
       </c>
       <c r="G3" s="16" t="n">
         <v>0.888</v>
@@ -7362,19 +7350,19 @@
         </is>
       </c>
       <c r="B4" s="19" t="n">
-        <v>100.43</v>
+        <v>99.47</v>
       </c>
       <c r="C4" s="20" t="n">
-        <v>0.176</v>
+        <v>0.165</v>
       </c>
       <c r="D4" s="20" t="n">
-        <v>-0.179</v>
+        <v>-0.187</v>
       </c>
       <c r="E4" s="16" t="n">
-        <v>39.3</v>
+        <v>33.2</v>
       </c>
       <c r="F4" s="20" t="n">
-        <v>-0.255</v>
+        <v>-0.262</v>
       </c>
       <c r="G4" s="16" t="n">
         <v>1.034</v>
@@ -7387,19 +7375,19 @@
         </is>
       </c>
       <c r="B5" s="19" t="n">
-        <v>28.06</v>
+        <v>26.89</v>
       </c>
       <c r="C5" s="20" t="n">
-        <v>-0</v>
+        <v>-0.004</v>
       </c>
       <c r="D5" s="20" t="n">
-        <v>0.191</v>
+        <v>0.141</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>-25.8</v>
+        <v>-21.9</v>
       </c>
       <c r="F5" s="20" t="n">
-        <v>-0.111</v>
+        <v>-0.149</v>
       </c>
       <c r="G5" s="16" t="n">
         <v>1.977</v>
@@ -7412,19 +7400,19 @@
         </is>
       </c>
       <c r="B6" s="19" t="n">
-        <v>14.31</v>
+        <v>14.57</v>
       </c>
       <c r="C6" s="20" t="n">
-        <v>-0.163</v>
+        <v>-0.149</v>
       </c>
       <c r="D6" s="20" t="n">
-        <v>-0.036</v>
+        <v>-0.019</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>-18.2</v>
+        <v>-19.4</v>
       </c>
       <c r="F6" s="20" t="n">
-        <v>-0.306</v>
+        <v>-0.293</v>
       </c>
       <c r="G6" s="16" t="n">
         <v>1.364</v>
@@ -7437,19 +7425,19 @@
         </is>
       </c>
       <c r="B7" s="19" t="n">
-        <v>81.64</v>
+        <v>82.94</v>
       </c>
       <c r="C7" s="20" t="n">
-        <v>0.203</v>
+        <v>0.235</v>
       </c>
       <c r="D7" s="20" t="n">
-        <v>-0.053</v>
+        <v>-0.035</v>
       </c>
       <c r="E7" s="16" t="n">
-        <v>22.5</v>
+        <v>19.9</v>
       </c>
       <c r="F7" s="20" t="n">
-        <v>-0.092</v>
+        <v>-0.078</v>
       </c>
       <c r="G7" s="16" t="n">
         <v>1.22</v>
@@ -7462,19 +7450,19 @@
         </is>
       </c>
       <c r="B8" s="19" t="n">
-        <v>57.84</v>
+        <v>55.74</v>
       </c>
       <c r="C8" s="20" t="n">
-        <v>0.357</v>
+        <v>0.325</v>
       </c>
       <c r="D8" s="20" t="n">
-        <v>-0.067</v>
+        <v>-0.09699999999999999</v>
       </c>
       <c r="E8" s="16" t="n">
-        <v>41.6</v>
+        <v>38.1</v>
       </c>
       <c r="F8" s="20" t="n">
-        <v>-0.162</v>
+        <v>-0.192</v>
       </c>
       <c r="G8" s="16" t="n">
         <v>1.453</v>
@@ -7487,19 +7475,19 @@
         </is>
       </c>
       <c r="B9" s="19" t="n">
-        <v>86.36</v>
+        <v>87.56999999999999</v>
       </c>
       <c r="C9" s="20" t="n">
-        <v>-0.215</v>
+        <v>-0.218</v>
       </c>
       <c r="D9" s="20" t="n">
-        <v>-0.229</v>
+        <v>-0.218</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>-2.2</v>
+        <v>-2.9</v>
       </c>
       <c r="F9" s="20" t="n">
-        <v>-0.271</v>
+        <v>-0.261</v>
       </c>
       <c r="G9" s="16" t="n">
         <v>0.66</v>
@@ -7512,19 +7500,19 @@
         </is>
       </c>
       <c r="B10" s="19" t="n">
-        <v>100.41</v>
+        <v>97.22</v>
       </c>
       <c r="C10" s="20" t="n">
-        <v>0.196</v>
+        <v>0.223</v>
       </c>
       <c r="D10" s="20" t="n">
-        <v>0.049</v>
+        <v>0.015</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>21.5</v>
+        <v>20.2</v>
       </c>
       <c r="F10" s="20" t="n">
-        <v>-0.118</v>
+        <v>-0.146</v>
       </c>
       <c r="G10" s="16" t="n">
         <v>1.376</v>
@@ -7537,19 +7525,19 @@
         </is>
       </c>
       <c r="B11" s="19" t="n">
-        <v>27.6</v>
+        <v>26.42</v>
       </c>
       <c r="C11" s="20" t="n">
-        <v>0.095</v>
+        <v>-0.005</v>
       </c>
       <c r="D11" s="20" t="n">
-        <v>0.011</v>
+        <v>-0.023</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>5</v>
+        <v>5.5</v>
       </c>
       <c r="F11" s="20" t="n">
-        <v>-0.157</v>
+        <v>-0.193</v>
       </c>
       <c r="G11" s="16" t="n">
         <v>1.412</v>
@@ -7562,19 +7550,19 @@
         </is>
       </c>
       <c r="B12" s="19" t="n">
-        <v>2.61</v>
+        <v>2.28</v>
       </c>
       <c r="C12" s="20" t="n">
-        <v>-0.352</v>
+        <v>-0.461</v>
       </c>
       <c r="D12" s="20" t="n">
-        <v>0.044</v>
+        <v>-0.08800000000000001</v>
       </c>
       <c r="E12" s="16" t="n">
-        <v>-53.3</v>
+        <v>-52.4</v>
       </c>
       <c r="F12" s="20" t="n">
-        <v>-0.473</v>
+        <v>-0.539</v>
       </c>
       <c r="G12" s="16" t="n">
         <v>1.327</v>
@@ -7587,19 +7575,19 @@
         </is>
       </c>
       <c r="B13" s="19" t="n">
-        <v>12.69</v>
+        <v>11.31</v>
       </c>
       <c r="C13" s="20" t="n">
-        <v>-0.248</v>
+        <v>-0.105</v>
       </c>
       <c r="D13" s="20" t="n">
-        <v>-0.237</v>
+        <v>-0.32</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>34.8</v>
+        <v>39.4</v>
       </c>
       <c r="F13" s="20" t="n">
-        <v>-0.388</v>
+        <v>-0.455</v>
       </c>
       <c r="G13" s="16" t="inlineStr">
         <is>
@@ -7614,19 +7602,19 @@
         </is>
       </c>
       <c r="B14" s="19" t="n">
-        <v>25.87</v>
+        <v>21.27</v>
       </c>
       <c r="C14" s="20" t="n">
-        <v>-0.317</v>
+        <v>-0.426</v>
       </c>
       <c r="D14" s="20" t="n">
-        <v>-0.275</v>
+        <v>-0.404</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>-31.9</v>
+        <v>-37.8</v>
       </c>
       <c r="F14" s="20" t="n">
-        <v>-0.47</v>
+        <v>-0.5639999999999999</v>
       </c>
       <c r="G14" s="16" t="n">
         <v>1.682</v>
@@ -7639,19 +7627,19 @@
         </is>
       </c>
       <c r="B15" s="19" t="n">
-        <v>108.37</v>
+        <v>103.57</v>
       </c>
       <c r="C15" s="20" t="n">
-        <v>-0.5429999999999999</v>
+        <v>-0.5639999999999999</v>
       </c>
       <c r="D15" s="20" t="n">
-        <v>-0.504</v>
+        <v>-0.525</v>
       </c>
       <c r="E15" s="16" t="n">
-        <v>-48</v>
+        <v>-60</v>
       </c>
       <c r="F15" s="20" t="n">
-        <v>-0.655</v>
+        <v>-0.67</v>
       </c>
       <c r="G15" s="16" t="n">
         <v>1.177</v>
@@ -7664,19 +7652,19 @@
         </is>
       </c>
       <c r="B16" s="19" t="n">
-        <v>20.25</v>
+        <v>21.45</v>
       </c>
       <c r="C16" s="20" t="n">
-        <v>0.893</v>
+        <v>0.9520000000000001</v>
       </c>
       <c r="D16" s="20" t="n">
-        <v>0.049</v>
+        <v>0.111</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>53.7</v>
+        <v>50.3</v>
       </c>
       <c r="F16" s="20" t="n">
-        <v>-0.106</v>
+        <v>-0.053</v>
       </c>
       <c r="G16" s="16" t="n">
         <v>1.552</v>
@@ -7689,19 +7677,19 @@
         </is>
       </c>
       <c r="B17" s="19" t="n">
-        <v>18.66</v>
+        <v>18</v>
       </c>
       <c r="C17" s="20" t="n">
-        <v>-0.07099999999999999</v>
+        <v>-0.2</v>
       </c>
       <c r="D17" s="20" t="n">
-        <v>-0.2</v>
+        <v>-0.228</v>
       </c>
       <c r="E17" s="16" t="n">
-        <v>-23</v>
+        <v>-30.1</v>
       </c>
       <c r="F17" s="20" t="n">
-        <v>-0.421</v>
+        <v>-0.441</v>
       </c>
       <c r="G17" s="16" t="n">
         <v>2.002</v>
@@ -7723,7 +7711,7 @@
         <v>-0.239</v>
       </c>
       <c r="E18" s="16" t="n">
-        <v>-283</v>
+        <v>-275.9</v>
       </c>
       <c r="F18" s="20" t="inlineStr">
         <is>
@@ -7743,19 +7731,19 @@
         </is>
       </c>
       <c r="B19" s="19" t="n">
-        <v>11.29</v>
+        <v>11.09</v>
       </c>
       <c r="C19" s="20" t="n">
-        <v>0.15</v>
+        <v>0.083</v>
       </c>
       <c r="D19" s="20" t="n">
-        <v>-0.006999999999999999</v>
+        <v>-0.025</v>
       </c>
       <c r="E19" s="16" t="n">
-        <v>0.4</v>
+        <v>-1.8</v>
       </c>
       <c r="F19" s="20" t="n">
-        <v>-0.152</v>
+        <v>-0.167</v>
       </c>
       <c r="G19" s="16" t="n">
         <v>1.07</v>
@@ -7768,19 +7756,19 @@
         </is>
       </c>
       <c r="B20" s="19" t="n">
-        <v>5.59</v>
+        <v>5.53</v>
       </c>
       <c r="C20" s="20" t="n">
-        <v>-0.006999999999999999</v>
+        <v>0.024</v>
       </c>
       <c r="D20" s="20" t="n">
-        <v>-0.256</v>
+        <v>-0.264</v>
       </c>
       <c r="E20" s="16" t="n">
-        <v>16.2</v>
+        <v>5.6</v>
       </c>
       <c r="F20" s="20" t="n">
-        <v>-0.449</v>
+        <v>-0.455</v>
       </c>
       <c r="G20" s="16" t="n">
         <v>0.603</v>

</xml_diff>